<commit_message>
Actualizacion adicional de plantillas de Revaluacion
</commit_message>
<xml_diff>
--- a/plantillas/REVALUACION_PROVEEDORES_TEMPLATE.xlsx
+++ b/plantillas/REVALUACION_PROVEEDORES_TEMPLATE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soporte y Desarrollo\Documents\NetBeansProjects\combinacion\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759454EA-ED19-48F7-A3F4-58272FCF1C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AFEEB51-C08D-4D40-A742-3045FF22C569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -320,7 +320,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -366,6 +366,11 @@
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -687,7 +692,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -754,18 +759,68 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -774,61 +829,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1919,34 +1929,34 @@
       <c r="K8" s="1"/>
     </row>
     <row r="9" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="27"/>
-      <c r="K9" s="28"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="29"/>
+      <c r="J9" s="29"/>
+      <c r="K9" s="30"/>
     </row>
     <row r="10" spans="2:27" ht="30" customHeight="1">
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="41" t="s">
+      <c r="C10" s="30"/>
+      <c r="D10" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="28"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="30"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
@@ -1965,20 +1975,20 @@
       <c r="AA10" s="1"/>
     </row>
     <row r="11" spans="2:27" ht="30" customHeight="1">
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="28"/>
-      <c r="D11" s="42" t="s">
+      <c r="C11" s="30"/>
+      <c r="D11" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="28"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
+      <c r="K11" s="30"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
@@ -1997,19 +2007,19 @@
       <c r="AA11" s="1"/>
     </row>
     <row r="12" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B12" s="41" t="s">
+      <c r="B12" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="31"/>
-      <c r="D12" s="41" t="s">
+      <c r="C12" s="37"/>
+      <c r="D12" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="46"/>
-      <c r="F12" s="31"/>
-      <c r="G12" s="37" t="s">
+      <c r="E12" s="27"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="H12" s="31"/>
+      <c r="H12" s="37"/>
       <c r="I12" s="3" t="s">
         <v>7</v>
       </c>
@@ -2037,13 +2047,13 @@
       <c r="AA12" s="1"/>
     </row>
     <row r="13" spans="2:27" ht="28.5" customHeight="1">
-      <c r="B13" s="47"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="47"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="47"/>
-      <c r="H13" s="49"/>
+      <c r="B13" s="41"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="53"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="41"/>
+      <c r="H13" s="42"/>
       <c r="I13" s="6" t="s">
         <v>10</v>
       </c>
@@ -2071,20 +2081,20 @@
       <c r="AA13" s="1"/>
     </row>
     <row r="14" spans="2:27" ht="30" customHeight="1">
-      <c r="B14" s="50" t="s">
+      <c r="B14" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="31"/>
-      <c r="D14" s="45" t="s">
+      <c r="C14" s="37"/>
+      <c r="D14" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
-      <c r="K14" s="28"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
+      <c r="K14" s="30"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
@@ -2103,20 +2113,20 @@
       <c r="AA14" s="1"/>
     </row>
     <row r="15" spans="2:27" ht="41.25" customHeight="1">
-      <c r="B15" s="41" t="s">
+      <c r="B15" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="41" t="s">
+      <c r="C15" s="30"/>
+      <c r="D15" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
-      <c r="K15" s="28"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
+      <c r="I15" s="29"/>
+      <c r="J15" s="29"/>
+      <c r="K15" s="30"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
@@ -2135,20 +2145,20 @@
       <c r="AA15" s="1"/>
     </row>
     <row r="16" spans="2:27" ht="30" customHeight="1">
-      <c r="B16" s="41" t="s">
+      <c r="B16" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="28"/>
-      <c r="D16" s="41" t="s">
+      <c r="C16" s="30"/>
+      <c r="D16" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="28"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+      <c r="J16" s="29"/>
+      <c r="K16" s="30"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
@@ -2167,20 +2177,20 @@
       <c r="AA16" s="1"/>
     </row>
     <row r="17" spans="2:27" ht="30" customHeight="1">
-      <c r="B17" s="29" t="s">
+      <c r="B17" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="40" t="s">
+      <c r="C17" s="30"/>
+      <c r="D17" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
-      <c r="K17" s="28"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="29"/>
+      <c r="I17" s="29"/>
+      <c r="J17" s="29"/>
+      <c r="K17" s="30"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
@@ -2199,20 +2209,20 @@
       <c r="AA17" s="1"/>
     </row>
     <row r="18" spans="2:27" ht="30" customHeight="1">
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="28"/>
-      <c r="D18" s="40" t="s">
+      <c r="C18" s="30"/>
+      <c r="D18" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
-      <c r="K18" s="28"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="29"/>
+      <c r="I18" s="29"/>
+      <c r="J18" s="29"/>
+      <c r="K18" s="30"/>
     </row>
     <row r="19" spans="2:27" ht="4.5" customHeight="1">
       <c r="B19" s="1"/>
@@ -2227,51 +2237,51 @@
       <c r="K19" s="1"/>
     </row>
     <row r="20" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B20" s="42" t="s">
+      <c r="B20" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="28"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="30"/>
     </row>
     <row r="21" spans="2:27" ht="30" customHeight="1">
-      <c r="B21" s="30" t="s">
+      <c r="B21" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="31"/>
-      <c r="D21" s="30" t="s">
+      <c r="C21" s="37"/>
+      <c r="D21" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="46"/>
-      <c r="F21" s="46"/>
-      <c r="G21" s="31"/>
-      <c r="H21" s="30" t="s">
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="I21" s="31"/>
-      <c r="J21" s="30" t="s">
+      <c r="I21" s="37"/>
+      <c r="J21" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="K21" s="31"/>
+      <c r="K21" s="37"/>
     </row>
     <row r="22" spans="2:27" ht="30" customHeight="1">
-      <c r="B22" s="41" t="s">
+      <c r="B22" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="31"/>
-      <c r="D22" s="41" t="s">
+      <c r="C22" s="37"/>
+      <c r="D22" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="42">
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="32">
         <v>60</v>
       </c>
       <c r="I22" s="6">
@@ -2280,57 +2290,58 @@
       <c r="J22" s="9">
         <v>30</v>
       </c>
-      <c r="K22" s="42">
+      <c r="K22" s="63">
+        <f>SUM(J22:J24)</f>
         <v>60</v>
       </c>
     </row>
     <row r="23" spans="2:27" ht="30" customHeight="1">
-      <c r="B23" s="51"/>
-      <c r="C23" s="52"/>
-      <c r="D23" s="41" t="s">
+      <c r="B23" s="39"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="43"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="33"/>
       <c r="I23" s="6">
         <v>15</v>
       </c>
       <c r="J23" s="9">
         <v>15</v>
       </c>
-      <c r="K23" s="43"/>
+      <c r="K23" s="64"/>
     </row>
     <row r="24" spans="2:27" ht="30" customHeight="1">
-      <c r="B24" s="47"/>
-      <c r="C24" s="49"/>
-      <c r="D24" s="41" t="s">
+      <c r="B24" s="41"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="44"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="34"/>
       <c r="I24" s="6">
         <v>15</v>
       </c>
       <c r="J24" s="9">
         <v>15</v>
       </c>
-      <c r="K24" s="44"/>
+      <c r="K24" s="65"/>
     </row>
     <row r="25" spans="2:27" ht="30" customHeight="1">
-      <c r="B25" s="57" t="s">
+      <c r="B25" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="C25" s="31"/>
-      <c r="D25" s="41" t="s">
+      <c r="C25" s="37"/>
+      <c r="D25" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
-      <c r="G25" s="28"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="30"/>
       <c r="H25" s="8">
         <v>10</v>
       </c>
@@ -2341,21 +2352,22 @@
         <v>10</v>
       </c>
       <c r="K25" s="6">
+        <f>SUM(J25)</f>
         <v>10</v>
       </c>
     </row>
     <row r="26" spans="2:27" ht="30" customHeight="1">
-      <c r="B26" s="41" t="s">
+      <c r="B26" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="C26" s="31"/>
-      <c r="D26" s="41" t="s">
+      <c r="C26" s="37"/>
+      <c r="D26" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="58">
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="46">
         <v>30</v>
       </c>
       <c r="I26" s="6">
@@ -2364,55 +2376,56 @@
       <c r="J26" s="9">
         <v>10</v>
       </c>
-      <c r="K26" s="42">
+      <c r="K26" s="32">
+        <f>SUM(J26:J28)</f>
         <v>30</v>
       </c>
     </row>
     <row r="27" spans="2:27" ht="30" customHeight="1">
-      <c r="B27" s="51"/>
-      <c r="C27" s="52"/>
-      <c r="D27" s="41" t="s">
+      <c r="B27" s="39"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="28"/>
-      <c r="H27" s="43"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="33"/>
       <c r="I27" s="6">
         <v>10</v>
       </c>
       <c r="J27" s="9">
         <v>10</v>
       </c>
-      <c r="K27" s="43"/>
+      <c r="K27" s="33"/>
     </row>
     <row r="28" spans="2:27" ht="42" customHeight="1">
-      <c r="B28" s="47"/>
-      <c r="C28" s="49"/>
-      <c r="D28" s="41" t="s">
+      <c r="B28" s="41"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="43"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="33"/>
       <c r="I28" s="6">
         <v>10</v>
       </c>
       <c r="J28" s="9">
         <v>10</v>
       </c>
-      <c r="K28" s="44"/>
+      <c r="K28" s="34"/>
     </row>
     <row r="29" spans="2:27" ht="30" customHeight="1">
-      <c r="B29" s="42" t="s">
+      <c r="B29" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="28"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="30"/>
       <c r="H29" s="6">
         <f>SUM(H22:H28)</f>
         <v>100</v>
@@ -2421,42 +2434,42 @@
         <f>SUM(I22:I28)</f>
         <v>100</v>
       </c>
-      <c r="J29" s="42">
+      <c r="J29" s="32">
         <f>SUM(K22:K28)</f>
         <v>100</v>
       </c>
-      <c r="K29" s="28"/>
+      <c r="K29" s="30"/>
     </row>
     <row r="30" spans="2:27" ht="30" customHeight="1">
-      <c r="B30" s="42" t="s">
+      <c r="B30" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="36" t="str">
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="29"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="31" t="str">
         <f>IF(J29&lt;65,B38,IF(J29&lt;75,B37,IF(J29&lt;90,B36,B35)))</f>
         <v>Satisfactorio</v>
       </c>
-      <c r="K30" s="28"/>
+      <c r="K30" s="30"/>
     </row>
     <row r="31" spans="2:27" ht="105" customHeight="1">
-      <c r="B31" s="26" t="s">
+      <c r="B31" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="27"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="28"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="29"/>
+      <c r="J31" s="29"/>
+      <c r="K31" s="30"/>
     </row>
     <row r="32" spans="2:27" ht="4.5" customHeight="1">
       <c r="B32" s="1"/>
@@ -2471,134 +2484,134 @@
       <c r="K32" s="1"/>
     </row>
     <row r="33" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B33" s="42" t="s">
+      <c r="B33" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="C33" s="27"/>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="27"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="27"/>
-      <c r="J33" s="27"/>
-      <c r="K33" s="28"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
+      <c r="J33" s="29"/>
+      <c r="K33" s="30"/>
     </row>
     <row r="34" spans="2:27" ht="30" customHeight="1">
-      <c r="B34" s="36" t="s">
+      <c r="B34" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="28"/>
-      <c r="D34" s="36" t="s">
+      <c r="C34" s="30"/>
+      <c r="D34" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="E34" s="28"/>
-      <c r="F34" s="32" t="s">
+      <c r="E34" s="30"/>
+      <c r="F34" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="G34" s="27"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="27"/>
-      <c r="J34" s="27"/>
-      <c r="K34" s="28"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
+      <c r="J34" s="29"/>
+      <c r="K34" s="30"/>
     </row>
     <row r="35" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B35" s="42" t="s">
+      <c r="B35" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="C35" s="28"/>
-      <c r="D35" s="37" t="s">
+      <c r="C35" s="30"/>
+      <c r="D35" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="E35" s="28"/>
-      <c r="F35" s="37" t="s">
+      <c r="E35" s="30"/>
+      <c r="F35" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="G35" s="27"/>
-      <c r="H35" s="27"/>
-      <c r="I35" s="27"/>
-      <c r="J35" s="27"/>
-      <c r="K35" s="28"/>
+      <c r="G35" s="29"/>
+      <c r="H35" s="29"/>
+      <c r="I35" s="29"/>
+      <c r="J35" s="29"/>
+      <c r="K35" s="30"/>
     </row>
     <row r="36" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B36" s="42" t="s">
+      <c r="B36" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="C36" s="28"/>
-      <c r="D36" s="37" t="s">
+      <c r="C36" s="30"/>
+      <c r="D36" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="28"/>
-      <c r="F36" s="37" t="s">
+      <c r="E36" s="30"/>
+      <c r="F36" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="G36" s="27"/>
-      <c r="H36" s="27"/>
-      <c r="I36" s="27"/>
-      <c r="J36" s="27"/>
-      <c r="K36" s="28"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="29"/>
+      <c r="J36" s="29"/>
+      <c r="K36" s="30"/>
     </row>
     <row r="37" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B37" s="42" t="s">
+      <c r="B37" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="C37" s="28"/>
-      <c r="D37" s="37" t="s">
+      <c r="C37" s="30"/>
+      <c r="D37" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="E37" s="28"/>
-      <c r="F37" s="37" t="s">
+      <c r="E37" s="30"/>
+      <c r="F37" s="44" t="s">
         <v>52</v>
       </c>
-      <c r="G37" s="27"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
-      <c r="J37" s="27"/>
-      <c r="K37" s="28"/>
+      <c r="G37" s="29"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="29"/>
+      <c r="J37" s="29"/>
+      <c r="K37" s="30"/>
     </row>
     <row r="38" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B38" s="42" t="s">
+      <c r="B38" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="C38" s="28"/>
-      <c r="D38" s="42" t="s">
+      <c r="C38" s="30"/>
+      <c r="D38" s="32" t="s">
         <v>54</v>
       </c>
-      <c r="E38" s="28"/>
-      <c r="F38" s="37" t="s">
+      <c r="E38" s="30"/>
+      <c r="F38" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="27"/>
-      <c r="J38" s="27"/>
-      <c r="K38" s="28"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="29"/>
+      <c r="J38" s="29"/>
+      <c r="K38" s="30"/>
     </row>
     <row r="39" spans="2:27" ht="4.5" customHeight="1">
-      <c r="B39" s="38"/>
-      <c r="C39" s="39"/>
+      <c r="B39" s="50"/>
+      <c r="C39" s="51"/>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
-      <c r="H39" s="38"/>
-      <c r="I39" s="39"/>
-      <c r="J39" s="39"/>
-      <c r="K39" s="39"/>
+      <c r="H39" s="50"/>
+      <c r="I39" s="51"/>
+      <c r="J39" s="51"/>
+      <c r="K39" s="51"/>
     </row>
     <row r="40" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B40" s="42" t="s">
+      <c r="B40" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="27"/>
-      <c r="J40" s="27"/>
-      <c r="K40" s="28"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="29"/>
+      <c r="I40" s="29"/>
+      <c r="J40" s="29"/>
+      <c r="K40" s="30"/>
     </row>
     <row r="41" spans="2:27" ht="22.5" customHeight="1">
       <c r="B41" s="60" t="s">
@@ -2632,127 +2645,127 @@
     </row>
     <row r="42" spans="2:27" ht="25.5" customHeight="1">
       <c r="B42" s="6"/>
-      <c r="C42" s="29" t="s">
+      <c r="C42" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="D42" s="27"/>
-      <c r="E42" s="27"/>
-      <c r="F42" s="27"/>
-      <c r="G42" s="27"/>
-      <c r="H42" s="27"/>
-      <c r="I42" s="27"/>
-      <c r="J42" s="27"/>
-      <c r="K42" s="28"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="29"/>
+      <c r="H42" s="29"/>
+      <c r="I42" s="29"/>
+      <c r="J42" s="29"/>
+      <c r="K42" s="30"/>
     </row>
     <row r="43" spans="2:27" ht="25.5" customHeight="1">
       <c r="B43" s="6"/>
-      <c r="C43" s="29" t="s">
+      <c r="C43" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="D43" s="27"/>
-      <c r="E43" s="27"/>
-      <c r="F43" s="27"/>
-      <c r="G43" s="27"/>
-      <c r="H43" s="27"/>
-      <c r="I43" s="27"/>
-      <c r="J43" s="27"/>
-      <c r="K43" s="28"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="29"/>
+      <c r="I43" s="29"/>
+      <c r="J43" s="29"/>
+      <c r="K43" s="30"/>
     </row>
     <row r="44" spans="2:27" ht="25.5" customHeight="1">
       <c r="B44" s="6"/>
-      <c r="C44" s="29" t="s">
+      <c r="C44" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="D44" s="27"/>
-      <c r="E44" s="27"/>
-      <c r="F44" s="27"/>
-      <c r="G44" s="27"/>
-      <c r="H44" s="27"/>
-      <c r="I44" s="27"/>
-      <c r="J44" s="27"/>
-      <c r="K44" s="28"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="29"/>
+      <c r="G44" s="29"/>
+      <c r="H44" s="29"/>
+      <c r="I44" s="29"/>
+      <c r="J44" s="29"/>
+      <c r="K44" s="30"/>
     </row>
     <row r="45" spans="2:27" ht="25.5" customHeight="1">
       <c r="B45" s="6"/>
-      <c r="C45" s="29" t="s">
+      <c r="C45" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="D45" s="27"/>
-      <c r="E45" s="27"/>
-      <c r="F45" s="27"/>
-      <c r="G45" s="27"/>
-      <c r="H45" s="27"/>
-      <c r="I45" s="27"/>
-      <c r="J45" s="27"/>
-      <c r="K45" s="28"/>
+      <c r="D45" s="29"/>
+      <c r="E45" s="29"/>
+      <c r="F45" s="29"/>
+      <c r="G45" s="29"/>
+      <c r="H45" s="29"/>
+      <c r="I45" s="29"/>
+      <c r="J45" s="29"/>
+      <c r="K45" s="30"/>
     </row>
     <row r="46" spans="2:27" ht="25.5" customHeight="1">
       <c r="B46" s="6"/>
-      <c r="C46" s="29" t="s">
+      <c r="C46" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="D46" s="27"/>
-      <c r="E46" s="27"/>
-      <c r="F46" s="27"/>
-      <c r="G46" s="27"/>
-      <c r="H46" s="27"/>
-      <c r="I46" s="27"/>
-      <c r="J46" s="27"/>
-      <c r="K46" s="28"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
+      <c r="H46" s="29"/>
+      <c r="I46" s="29"/>
+      <c r="J46" s="29"/>
+      <c r="K46" s="30"/>
     </row>
     <row r="47" spans="2:27" ht="25.5" customHeight="1">
       <c r="B47" s="6"/>
-      <c r="C47" s="29" t="s">
+      <c r="C47" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="D47" s="27"/>
-      <c r="E47" s="27"/>
-      <c r="F47" s="27"/>
-      <c r="G47" s="27"/>
-      <c r="H47" s="27"/>
-      <c r="I47" s="27"/>
-      <c r="J47" s="27"/>
-      <c r="K47" s="28"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="29"/>
+      <c r="F47" s="29"/>
+      <c r="G47" s="29"/>
+      <c r="H47" s="29"/>
+      <c r="I47" s="29"/>
+      <c r="J47" s="29"/>
+      <c r="K47" s="30"/>
     </row>
     <row r="48" spans="2:27" ht="89.25" customHeight="1">
       <c r="B48" s="6"/>
-      <c r="C48" s="26" t="s">
+      <c r="C48" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="D48" s="27"/>
-      <c r="E48" s="27"/>
-      <c r="F48" s="27"/>
-      <c r="G48" s="27"/>
-      <c r="H48" s="27"/>
-      <c r="I48" s="27"/>
-      <c r="J48" s="27"/>
-      <c r="K48" s="28"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="29"/>
+      <c r="G48" s="29"/>
+      <c r="H48" s="29"/>
+      <c r="I48" s="29"/>
+      <c r="J48" s="29"/>
+      <c r="K48" s="30"/>
     </row>
     <row r="49" spans="2:27" ht="4.5" customHeight="1">
-      <c r="B49" s="38"/>
-      <c r="C49" s="39"/>
+      <c r="B49" s="50"/>
+      <c r="C49" s="51"/>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
-      <c r="H49" s="38"/>
-      <c r="I49" s="39"/>
-      <c r="J49" s="39"/>
-      <c r="K49" s="39"/>
+      <c r="H49" s="50"/>
+      <c r="I49" s="51"/>
+      <c r="J49" s="51"/>
+      <c r="K49" s="51"/>
     </row>
     <row r="50" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B50" s="33" t="s">
+      <c r="B50" s="57" t="s">
         <v>64</v>
       </c>
-      <c r="C50" s="34"/>
-      <c r="D50" s="34"/>
-      <c r="E50" s="34"/>
-      <c r="F50" s="34"/>
-      <c r="G50" s="34"/>
-      <c r="H50" s="34"/>
-      <c r="I50" s="34"/>
-      <c r="J50" s="34"/>
-      <c r="K50" s="35"/>
+      <c r="C50" s="58"/>
+      <c r="D50" s="58"/>
+      <c r="E50" s="58"/>
+      <c r="F50" s="58"/>
+      <c r="G50" s="58"/>
+      <c r="H50" s="58"/>
+      <c r="I50" s="58"/>
+      <c r="J50" s="58"/>
+      <c r="K50" s="59"/>
     </row>
     <row r="51" spans="2:27" ht="18" customHeight="1">
       <c r="B51" s="15"/>
@@ -2779,10 +2792,10 @@
       <c r="K52" s="20"/>
     </row>
     <row r="53" spans="2:27" ht="42" customHeight="1">
-      <c r="B53" s="56"/>
-      <c r="C53" s="48"/>
-      <c r="D53" s="48"/>
-      <c r="E53" s="48"/>
+      <c r="B53" s="52"/>
+      <c r="C53" s="53"/>
+      <c r="D53" s="53"/>
+      <c r="E53" s="53"/>
       <c r="F53" s="21"/>
       <c r="G53" s="22"/>
       <c r="H53" s="22"/>
@@ -2791,12 +2804,12 @@
       <c r="K53" s="23"/>
     </row>
     <row r="54" spans="2:27" ht="41.45" customHeight="1">
-      <c r="B54" s="59" t="s">
+      <c r="B54" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="C54" s="46"/>
-      <c r="D54" s="46"/>
-      <c r="E54" s="46"/>
+      <c r="C54" s="27"/>
+      <c r="D54" s="27"/>
+      <c r="E54" s="27"/>
       <c r="F54" s="21"/>
       <c r="G54" s="22"/>
       <c r="H54" s="22"/>
@@ -2833,18 +2846,18 @@
       <c r="AA55" s="10"/>
     </row>
     <row r="56" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B56" s="53" t="s">
+      <c r="B56" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="C56" s="54"/>
-      <c r="D56" s="54"/>
-      <c r="E56" s="54"/>
-      <c r="F56" s="54"/>
-      <c r="G56" s="54"/>
-      <c r="H56" s="54"/>
-      <c r="I56" s="54"/>
-      <c r="J56" s="54"/>
-      <c r="K56" s="55"/>
+      <c r="C56" s="48"/>
+      <c r="D56" s="48"/>
+      <c r="E56" s="48"/>
+      <c r="F56" s="48"/>
+      <c r="G56" s="48"/>
+      <c r="H56" s="48"/>
+      <c r="I56" s="48"/>
+      <c r="J56" s="48"/>
+      <c r="K56" s="49"/>
     </row>
     <row r="57" spans="2:27" ht="6.75" customHeight="1">
       <c r="B57" s="11"/>
@@ -3887,6 +3900,65 @@
     <row r="996" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="75">
+    <mergeCell ref="C48:K48"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="F34:K34"/>
+    <mergeCell ref="B50:K50"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="F37:K37"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="B41:K41"/>
+    <mergeCell ref="C45:K45"/>
+    <mergeCell ref="H49:K49"/>
+    <mergeCell ref="D18:K18"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="K22:K24"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D14:K14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D12:F13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="F36:K36"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="B22:C24"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="K26:K28"/>
+    <mergeCell ref="B56:K56"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="C44:K44"/>
+    <mergeCell ref="C47:K47"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B33:K33"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="F38:K38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:K10"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="F35:K35"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B12:C13"/>
+    <mergeCell ref="D15:K15"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="G12:H13"/>
+    <mergeCell ref="D17:K17"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="D28:G28"/>
+    <mergeCell ref="D11:K11"/>
     <mergeCell ref="B54:E54"/>
     <mergeCell ref="C43:K43"/>
     <mergeCell ref="D34:E34"/>
@@ -3903,65 +3975,6 @@
     <mergeCell ref="C42:K42"/>
     <mergeCell ref="B26:C28"/>
     <mergeCell ref="D25:G25"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:K10"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="F35:K35"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B12:C13"/>
-    <mergeCell ref="D15:K15"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="G12:H13"/>
-    <mergeCell ref="D17:K17"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="D28:G28"/>
-    <mergeCell ref="D11:K11"/>
-    <mergeCell ref="B56:K56"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="C44:K44"/>
-    <mergeCell ref="C47:K47"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="B33:K33"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="F38:K38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B53:E53"/>
-    <mergeCell ref="F36:K36"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="B22:C24"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="K26:K28"/>
-    <mergeCell ref="D14:K14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D12:F13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="C48:K48"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="F34:K34"/>
-    <mergeCell ref="B50:K50"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="F37:K37"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="B41:K41"/>
-    <mergeCell ref="C45:K45"/>
-    <mergeCell ref="H49:K49"/>
-    <mergeCell ref="D18:K18"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="K22:K24"/>
-    <mergeCell ref="D38:E38"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.78740157480314965" bottom="0.78740157480314965" header="0" footer="0"/>
@@ -3969,6 +3982,9 @@
   <headerFooter>
     <oddFooter>&amp;LEste documento es propiedad de la Administración Central del Distrito de Santiago de Cali. Prohibida su alteración o modificación por cualquier medio, sin previa autorización del Alcalde.&amp;RPágina &amp;P de</oddFooter>
   </headerFooter>
+  <ignoredErrors>
+    <ignoredError sqref="K26 K22" formulaRange="1"/>
+  </ignoredErrors>
   <drawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">

</xml_diff>

<commit_message>
Actualizar plantilla Excel con variables separadas para fecha suscripcion y fecha generacion
</commit_message>
<xml_diff>
--- a/plantillas/REVALUACION_PROVEEDORES_TEMPLATE.xlsx
+++ b/plantillas/REVALUACION_PROVEEDORES_TEMPLATE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soporte y Desarrollo\Documents\NetBeansProjects\combinacion\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AFEEB51-C08D-4D40-A742-3045FF22C569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AAA1580-3B95-4DBC-B44E-8EA902A35950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,15 +56,6 @@
   </si>
   <si>
     <t>AÑO</t>
-  </si>
-  <si>
-    <t>${DIA}</t>
-  </si>
-  <si>
-    <t>${MES}</t>
-  </si>
-  <si>
-    <t>${ANIO}</t>
   </si>
   <si>
     <t>VALOR:</t>
@@ -311,6 +302,15 @@
       </rPr>
       <t xml:space="preserve"> la casilla correspondiente</t>
     </r>
+  </si>
+  <si>
+    <t>${DIA_SUSC}</t>
+  </si>
+  <si>
+    <t>${MES_SUSC}</t>
+  </si>
+  <si>
+    <t>${ANIO_SUSC}</t>
   </si>
 </sst>
 </file>
@@ -759,68 +759,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -829,16 +779,66 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1929,34 +1929,34 @@
       <c r="K8" s="1"/>
     </row>
     <row r="9" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="29"/>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="29"/>
-      <c r="K9" s="30"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="28"/>
     </row>
     <row r="10" spans="2:27" ht="30" customHeight="1">
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="30"/>
-      <c r="D10" s="35" t="s">
-        <v>81</v>
-      </c>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
-      <c r="K10" s="30"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="44" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
+      <c r="K10" s="28"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
@@ -1975,20 +1975,20 @@
       <c r="AA10" s="1"/>
     </row>
     <row r="11" spans="2:27" ht="30" customHeight="1">
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="30"/>
-      <c r="D11" s="32" t="s">
+      <c r="C11" s="28"/>
+      <c r="D11" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="29"/>
-      <c r="K11" s="30"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
+      <c r="K11" s="28"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
@@ -2007,19 +2007,19 @@
       <c r="AA11" s="1"/>
     </row>
     <row r="12" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B12" s="35" t="s">
+      <c r="B12" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="37"/>
-      <c r="D12" s="35" t="s">
+      <c r="C12" s="31"/>
+      <c r="D12" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="27"/>
-      <c r="F12" s="37"/>
-      <c r="G12" s="44" t="s">
+      <c r="E12" s="50"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="H12" s="37"/>
+      <c r="H12" s="31"/>
       <c r="I12" s="3" t="s">
         <v>7</v>
       </c>
@@ -2047,21 +2047,21 @@
       <c r="AA12" s="1"/>
     </row>
     <row r="13" spans="2:27" ht="28.5" customHeight="1">
-      <c r="B13" s="41"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="53"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="42"/>
+      <c r="B13" s="51"/>
+      <c r="C13" s="53"/>
+      <c r="D13" s="51"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="53"/>
+      <c r="G13" s="51"/>
+      <c r="H13" s="53"/>
       <c r="I13" s="6" t="s">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>11</v>
+        <v>81</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
@@ -2081,20 +2081,20 @@
       <c r="AA13" s="1"/>
     </row>
     <row r="14" spans="2:27" ht="30" customHeight="1">
-      <c r="B14" s="55" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="37"/>
-      <c r="D14" s="54" t="s">
-        <v>14</v>
-      </c>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="29"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="29"/>
-      <c r="K14" s="30"/>
+      <c r="B14" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="31"/>
+      <c r="D14" s="49" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
+      <c r="K14" s="28"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
@@ -2113,20 +2113,20 @@
       <c r="AA14" s="1"/>
     </row>
     <row r="15" spans="2:27" ht="41.25" customHeight="1">
-      <c r="B15" s="35" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="30"/>
-      <c r="D15" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="29"/>
-      <c r="H15" s="29"/>
-      <c r="I15" s="29"/>
-      <c r="J15" s="29"/>
-      <c r="K15" s="30"/>
+      <c r="B15" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="28"/>
+      <c r="D15" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="28"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
@@ -2145,20 +2145,20 @@
       <c r="AA15" s="1"/>
     </row>
     <row r="16" spans="2:27" ht="30" customHeight="1">
-      <c r="B16" s="35" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="30"/>
-      <c r="D16" s="35" t="s">
-        <v>18</v>
-      </c>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="29"/>
-      <c r="H16" s="29"/>
-      <c r="I16" s="29"/>
-      <c r="J16" s="29"/>
-      <c r="K16" s="30"/>
+      <c r="B16" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="28"/>
+      <c r="D16" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="28"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
@@ -2177,20 +2177,20 @@
       <c r="AA16" s="1"/>
     </row>
     <row r="17" spans="2:27" ht="30" customHeight="1">
-      <c r="B17" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" s="30"/>
-      <c r="D17" s="45" t="s">
-        <v>20</v>
-      </c>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
-      <c r="G17" s="29"/>
-      <c r="H17" s="29"/>
-      <c r="I17" s="29"/>
-      <c r="J17" s="29"/>
-      <c r="K17" s="30"/>
+      <c r="B17" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="28"/>
+      <c r="D17" s="43" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="28"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
@@ -2209,20 +2209,20 @@
       <c r="AA17" s="1"/>
     </row>
     <row r="18" spans="2:27" ht="30" customHeight="1">
-      <c r="B18" s="35" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="30"/>
-      <c r="D18" s="45" t="s">
-        <v>22</v>
-      </c>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="29"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="29"/>
-      <c r="J18" s="29"/>
-      <c r="K18" s="30"/>
+      <c r="B18" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="28"/>
+      <c r="D18" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="28"/>
     </row>
     <row r="19" spans="2:27" ht="4.5" customHeight="1">
       <c r="B19" s="1"/>
@@ -2237,51 +2237,51 @@
       <c r="K19" s="1"/>
     </row>
     <row r="20" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="28"/>
+    </row>
+    <row r="21" spans="2:27" ht="30" customHeight="1">
+      <c r="B21" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="31"/>
+      <c r="D21" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="50"/>
+      <c r="F21" s="50"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="29"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="29"/>
-      <c r="J20" s="29"/>
-      <c r="K20" s="30"/>
-    </row>
-    <row r="21" spans="2:27" ht="30" customHeight="1">
-      <c r="B21" s="36" t="s">
+      <c r="I21" s="31"/>
+      <c r="J21" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="37"/>
-      <c r="D21" s="36" t="s">
+      <c r="K21" s="31"/>
+    </row>
+    <row r="22" spans="2:27" ht="30" customHeight="1">
+      <c r="B22" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="36" t="s">
+      <c r="C22" s="31"/>
+      <c r="D22" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="I21" s="37"/>
-      <c r="J21" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="K21" s="37"/>
-    </row>
-    <row r="22" spans="2:27" ht="30" customHeight="1">
-      <c r="B22" s="35" t="s">
-        <v>28</v>
-      </c>
-      <c r="C22" s="37"/>
-      <c r="D22" s="35" t="s">
-        <v>29</v>
-      </c>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="32">
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="48">
         <v>60</v>
       </c>
       <c r="I22" s="6">
@@ -2290,58 +2290,58 @@
       <c r="J22" s="9">
         <v>30</v>
       </c>
-      <c r="K22" s="63">
+      <c r="K22" s="45">
         <f>SUM(J22:J24)</f>
         <v>60</v>
       </c>
     </row>
     <row r="23" spans="2:27" ht="30" customHeight="1">
-      <c r="B23" s="39"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="33"/>
+      <c r="B23" s="55"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="57"/>
       <c r="I23" s="6">
         <v>15</v>
       </c>
       <c r="J23" s="9">
         <v>15</v>
       </c>
-      <c r="K23" s="64"/>
+      <c r="K23" s="46"/>
     </row>
     <row r="24" spans="2:27" ht="30" customHeight="1">
-      <c r="B24" s="41"/>
-      <c r="C24" s="42"/>
-      <c r="D24" s="35" t="s">
-        <v>31</v>
-      </c>
-      <c r="E24" s="29"/>
-      <c r="F24" s="29"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="34"/>
+      <c r="B24" s="51"/>
+      <c r="C24" s="53"/>
+      <c r="D24" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="28"/>
+      <c r="H24" s="58"/>
       <c r="I24" s="6">
         <v>15</v>
       </c>
       <c r="J24" s="9">
         <v>15</v>
       </c>
-      <c r="K24" s="65"/>
+      <c r="K24" s="47"/>
     </row>
     <row r="25" spans="2:27" ht="30" customHeight="1">
-      <c r="B25" s="43" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25" s="37"/>
-      <c r="D25" s="35" t="s">
-        <v>33</v>
-      </c>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="30"/>
+      <c r="B25" s="63" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="31"/>
+      <c r="D25" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="28"/>
       <c r="H25" s="8">
         <v>10</v>
       </c>
@@ -2357,17 +2357,17 @@
       </c>
     </row>
     <row r="26" spans="2:27" ht="30" customHeight="1">
-      <c r="B26" s="35" t="s">
-        <v>34</v>
-      </c>
-      <c r="C26" s="37"/>
-      <c r="D26" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="46">
+      <c r="B26" s="44" t="s">
+        <v>31</v>
+      </c>
+      <c r="C26" s="31"/>
+      <c r="D26" s="44" t="s">
+        <v>32</v>
+      </c>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="28"/>
+      <c r="H26" s="64">
         <v>30</v>
       </c>
       <c r="I26" s="6">
@@ -2376,56 +2376,56 @@
       <c r="J26" s="9">
         <v>10</v>
       </c>
-      <c r="K26" s="32">
+      <c r="K26" s="48">
         <f>SUM(J26:J28)</f>
         <v>30</v>
       </c>
     </row>
     <row r="27" spans="2:27" ht="30" customHeight="1">
-      <c r="B27" s="39"/>
-      <c r="C27" s="40"/>
-      <c r="D27" s="35" t="s">
-        <v>36</v>
-      </c>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="33"/>
+      <c r="B27" s="55"/>
+      <c r="C27" s="56"/>
+      <c r="D27" s="44" t="s">
+        <v>33</v>
+      </c>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="57"/>
       <c r="I27" s="6">
         <v>10</v>
       </c>
       <c r="J27" s="9">
         <v>10</v>
       </c>
-      <c r="K27" s="33"/>
+      <c r="K27" s="57"/>
     </row>
     <row r="28" spans="2:27" ht="42" customHeight="1">
-      <c r="B28" s="41"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="33"/>
+      <c r="B28" s="51"/>
+      <c r="C28" s="53"/>
+      <c r="D28" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="57"/>
       <c r="I28" s="6">
         <v>10</v>
       </c>
       <c r="J28" s="9">
         <v>10</v>
       </c>
-      <c r="K28" s="34"/>
+      <c r="K28" s="58"/>
     </row>
     <row r="29" spans="2:27" ht="30" customHeight="1">
-      <c r="B29" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="30"/>
+      <c r="B29" s="48" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="28"/>
       <c r="H29" s="6">
         <f>SUM(H22:H28)</f>
         <v>100</v>
@@ -2434,42 +2434,42 @@
         <f>SUM(I22:I28)</f>
         <v>100</v>
       </c>
-      <c r="J29" s="32">
+      <c r="J29" s="48">
         <f>SUM(K22:K28)</f>
         <v>100</v>
       </c>
-      <c r="K29" s="30"/>
+      <c r="K29" s="28"/>
     </row>
     <row r="30" spans="2:27" ht="30" customHeight="1">
-      <c r="B30" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="29"/>
-      <c r="G30" s="29"/>
-      <c r="H30" s="29"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="31" t="str">
+      <c r="B30" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="36" t="str">
         <f>IF(J29&lt;65,B38,IF(J29&lt;75,B37,IF(J29&lt;90,B36,B35)))</f>
         <v>Satisfactorio</v>
       </c>
-      <c r="K30" s="30"/>
+      <c r="K30" s="28"/>
     </row>
     <row r="31" spans="2:27" ht="105" customHeight="1">
-      <c r="B31" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="29"/>
-      <c r="F31" s="29"/>
-      <c r="G31" s="29"/>
-      <c r="H31" s="29"/>
-      <c r="I31" s="29"/>
-      <c r="J31" s="29"/>
-      <c r="K31" s="30"/>
+      <c r="B31" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31" s="27"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="27"/>
+      <c r="J31" s="27"/>
+      <c r="K31" s="28"/>
     </row>
     <row r="32" spans="2:27" ht="4.5" customHeight="1">
       <c r="B32" s="1"/>
@@ -2484,148 +2484,148 @@
       <c r="K32" s="1"/>
     </row>
     <row r="33" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B33" s="32" t="s">
+      <c r="B33" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" s="27"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="27"/>
+      <c r="J33" s="27"/>
+      <c r="K33" s="28"/>
+    </row>
+    <row r="34" spans="2:27" ht="30" customHeight="1">
+      <c r="B34" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="C34" s="28"/>
+      <c r="D34" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="E34" s="28"/>
+      <c r="F34" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
+      <c r="I34" s="27"/>
+      <c r="J34" s="27"/>
+      <c r="K34" s="28"/>
+    </row>
+    <row r="35" spans="2:27" ht="52.5" customHeight="1">
+      <c r="B35" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="29"/>
-      <c r="F33" s="29"/>
-      <c r="G33" s="29"/>
-      <c r="H33" s="29"/>
-      <c r="I33" s="29"/>
-      <c r="J33" s="29"/>
-      <c r="K33" s="30"/>
-    </row>
-    <row r="34" spans="2:27" ht="30" customHeight="1">
-      <c r="B34" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="C34" s="30"/>
-      <c r="D34" s="31" t="s">
+      <c r="C35" s="28"/>
+      <c r="D35" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="E34" s="30"/>
-      <c r="F34" s="56" t="s">
+      <c r="E35" s="28"/>
+      <c r="F35" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="G34" s="29"/>
-      <c r="H34" s="29"/>
-      <c r="I34" s="29"/>
-      <c r="J34" s="29"/>
-      <c r="K34" s="30"/>
-    </row>
-    <row r="35" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B35" s="32" t="s">
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="27"/>
+      <c r="J35" s="27"/>
+      <c r="K35" s="28"/>
+    </row>
+    <row r="36" spans="2:27" ht="52.5" customHeight="1">
+      <c r="B36" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="C35" s="30"/>
-      <c r="D35" s="44" t="s">
+      <c r="C36" s="28"/>
+      <c r="D36" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="E35" s="30"/>
-      <c r="F35" s="44" t="s">
+      <c r="E36" s="28"/>
+      <c r="F36" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="G35" s="29"/>
-      <c r="H35" s="29"/>
-      <c r="I35" s="29"/>
-      <c r="J35" s="29"/>
-      <c r="K35" s="30"/>
-    </row>
-    <row r="36" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B36" s="32" t="s">
+      <c r="G36" s="27"/>
+      <c r="H36" s="27"/>
+      <c r="I36" s="27"/>
+      <c r="J36" s="27"/>
+      <c r="K36" s="28"/>
+    </row>
+    <row r="37" spans="2:27" ht="52.5" customHeight="1">
+      <c r="B37" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="C36" s="30"/>
-      <c r="D36" s="44" t="s">
+      <c r="C37" s="28"/>
+      <c r="D37" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="30"/>
-      <c r="F36" s="44" t="s">
+      <c r="E37" s="28"/>
+      <c r="F37" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="G36" s="29"/>
-      <c r="H36" s="29"/>
-      <c r="I36" s="29"/>
-      <c r="J36" s="29"/>
-      <c r="K36" s="30"/>
-    </row>
-    <row r="37" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B37" s="32" t="s">
+      <c r="G37" s="27"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="27"/>
+      <c r="J37" s="27"/>
+      <c r="K37" s="28"/>
+    </row>
+    <row r="38" spans="2:27" ht="52.5" customHeight="1">
+      <c r="B38" s="48" t="s">
         <v>50</v>
       </c>
-      <c r="C37" s="30"/>
-      <c r="D37" s="44" t="s">
+      <c r="C38" s="28"/>
+      <c r="D38" s="48" t="s">
         <v>51</v>
       </c>
-      <c r="E37" s="30"/>
-      <c r="F37" s="44" t="s">
+      <c r="E38" s="28"/>
+      <c r="F38" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="G37" s="29"/>
-      <c r="H37" s="29"/>
-      <c r="I37" s="29"/>
-      <c r="J37" s="29"/>
-      <c r="K37" s="30"/>
-    </row>
-    <row r="38" spans="2:27" ht="52.5" customHeight="1">
-      <c r="B38" s="32" t="s">
-        <v>53</v>
-      </c>
-      <c r="C38" s="30"/>
-      <c r="D38" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="E38" s="30"/>
-      <c r="F38" s="44" t="s">
-        <v>55</v>
-      </c>
-      <c r="G38" s="29"/>
-      <c r="H38" s="29"/>
-      <c r="I38" s="29"/>
-      <c r="J38" s="29"/>
-      <c r="K38" s="30"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="27"/>
+      <c r="I38" s="27"/>
+      <c r="J38" s="27"/>
+      <c r="K38" s="28"/>
     </row>
     <row r="39" spans="2:27" ht="4.5" customHeight="1">
-      <c r="B39" s="50"/>
-      <c r="C39" s="51"/>
+      <c r="B39" s="41"/>
+      <c r="C39" s="42"/>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
-      <c r="H39" s="50"/>
-      <c r="I39" s="51"/>
-      <c r="J39" s="51"/>
-      <c r="K39" s="51"/>
+      <c r="H39" s="41"/>
+      <c r="I39" s="42"/>
+      <c r="J39" s="42"/>
+      <c r="K39" s="42"/>
     </row>
     <row r="40" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B40" s="32" t="s">
-        <v>56</v>
-      </c>
-      <c r="C40" s="29"/>
-      <c r="D40" s="29"/>
-      <c r="E40" s="29"/>
-      <c r="F40" s="29"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="29"/>
-      <c r="K40" s="30"/>
+      <c r="B40" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="28"/>
     </row>
     <row r="41" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B41" s="60" t="s">
-        <v>82</v>
-      </c>
-      <c r="C41" s="61"/>
-      <c r="D41" s="61"/>
-      <c r="E41" s="61"/>
-      <c r="F41" s="61"/>
-      <c r="G41" s="61"/>
-      <c r="H41" s="61"/>
-      <c r="I41" s="61"/>
-      <c r="J41" s="61"/>
-      <c r="K41" s="62"/>
+      <c r="B41" s="38" t="s">
+        <v>79</v>
+      </c>
+      <c r="C41" s="39"/>
+      <c r="D41" s="39"/>
+      <c r="E41" s="39"/>
+      <c r="F41" s="39"/>
+      <c r="G41" s="39"/>
+      <c r="H41" s="39"/>
+      <c r="I41" s="39"/>
+      <c r="J41" s="39"/>
+      <c r="K41" s="40"/>
       <c r="L41" s="10"/>
       <c r="M41" s="10"/>
       <c r="N41" s="10"/>
@@ -2645,127 +2645,127 @@
     </row>
     <row r="42" spans="2:27" ht="25.5" customHeight="1">
       <c r="B42" s="6"/>
-      <c r="C42" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="D42" s="29"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
-      <c r="H42" s="29"/>
-      <c r="I42" s="29"/>
-      <c r="J42" s="29"/>
-      <c r="K42" s="30"/>
+      <c r="C42" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="D42" s="27"/>
+      <c r="E42" s="27"/>
+      <c r="F42" s="27"/>
+      <c r="G42" s="27"/>
+      <c r="H42" s="27"/>
+      <c r="I42" s="27"/>
+      <c r="J42" s="27"/>
+      <c r="K42" s="28"/>
     </row>
     <row r="43" spans="2:27" ht="25.5" customHeight="1">
       <c r="B43" s="6"/>
-      <c r="C43" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="D43" s="29"/>
-      <c r="E43" s="29"/>
-      <c r="F43" s="29"/>
-      <c r="G43" s="29"/>
-      <c r="H43" s="29"/>
-      <c r="I43" s="29"/>
-      <c r="J43" s="29"/>
-      <c r="K43" s="30"/>
+      <c r="C43" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="D43" s="27"/>
+      <c r="E43" s="27"/>
+      <c r="F43" s="27"/>
+      <c r="G43" s="27"/>
+      <c r="H43" s="27"/>
+      <c r="I43" s="27"/>
+      <c r="J43" s="27"/>
+      <c r="K43" s="28"/>
     </row>
     <row r="44" spans="2:27" ht="25.5" customHeight="1">
       <c r="B44" s="6"/>
-      <c r="C44" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="D44" s="29"/>
-      <c r="E44" s="29"/>
-      <c r="F44" s="29"/>
-      <c r="G44" s="29"/>
-      <c r="H44" s="29"/>
-      <c r="I44" s="29"/>
-      <c r="J44" s="29"/>
-      <c r="K44" s="30"/>
+      <c r="C44" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="D44" s="27"/>
+      <c r="E44" s="27"/>
+      <c r="F44" s="27"/>
+      <c r="G44" s="27"/>
+      <c r="H44" s="27"/>
+      <c r="I44" s="27"/>
+      <c r="J44" s="27"/>
+      <c r="K44" s="28"/>
     </row>
     <row r="45" spans="2:27" ht="25.5" customHeight="1">
       <c r="B45" s="6"/>
-      <c r="C45" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="D45" s="29"/>
-      <c r="E45" s="29"/>
-      <c r="F45" s="29"/>
-      <c r="G45" s="29"/>
-      <c r="H45" s="29"/>
-      <c r="I45" s="29"/>
-      <c r="J45" s="29"/>
-      <c r="K45" s="30"/>
+      <c r="C45" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="D45" s="27"/>
+      <c r="E45" s="27"/>
+      <c r="F45" s="27"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="27"/>
+      <c r="I45" s="27"/>
+      <c r="J45" s="27"/>
+      <c r="K45" s="28"/>
     </row>
     <row r="46" spans="2:27" ht="25.5" customHeight="1">
       <c r="B46" s="6"/>
-      <c r="C46" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="D46" s="29"/>
-      <c r="E46" s="29"/>
-      <c r="F46" s="29"/>
-      <c r="G46" s="29"/>
-      <c r="H46" s="29"/>
-      <c r="I46" s="29"/>
-      <c r="J46" s="29"/>
-      <c r="K46" s="30"/>
+      <c r="C46" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27"/>
+      <c r="H46" s="27"/>
+      <c r="I46" s="27"/>
+      <c r="J46" s="27"/>
+      <c r="K46" s="28"/>
     </row>
     <row r="47" spans="2:27" ht="25.5" customHeight="1">
       <c r="B47" s="6"/>
-      <c r="C47" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="D47" s="29"/>
-      <c r="E47" s="29"/>
-      <c r="F47" s="29"/>
-      <c r="G47" s="29"/>
-      <c r="H47" s="29"/>
-      <c r="I47" s="29"/>
-      <c r="J47" s="29"/>
-      <c r="K47" s="30"/>
+      <c r="C47" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="D47" s="27"/>
+      <c r="E47" s="27"/>
+      <c r="F47" s="27"/>
+      <c r="G47" s="27"/>
+      <c r="H47" s="27"/>
+      <c r="I47" s="27"/>
+      <c r="J47" s="27"/>
+      <c r="K47" s="28"/>
     </row>
     <row r="48" spans="2:27" ht="89.25" customHeight="1">
       <c r="B48" s="6"/>
-      <c r="C48" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="D48" s="29"/>
-      <c r="E48" s="29"/>
-      <c r="F48" s="29"/>
-      <c r="G48" s="29"/>
-      <c r="H48" s="29"/>
-      <c r="I48" s="29"/>
-      <c r="J48" s="29"/>
-      <c r="K48" s="30"/>
+      <c r="C48" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="D48" s="27"/>
+      <c r="E48" s="27"/>
+      <c r="F48" s="27"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="27"/>
+      <c r="I48" s="27"/>
+      <c r="J48" s="27"/>
+      <c r="K48" s="28"/>
     </row>
     <row r="49" spans="2:27" ht="4.5" customHeight="1">
-      <c r="B49" s="50"/>
-      <c r="C49" s="51"/>
+      <c r="B49" s="41"/>
+      <c r="C49" s="42"/>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
-      <c r="H49" s="50"/>
-      <c r="I49" s="51"/>
-      <c r="J49" s="51"/>
-      <c r="K49" s="51"/>
+      <c r="H49" s="41"/>
+      <c r="I49" s="42"/>
+      <c r="J49" s="42"/>
+      <c r="K49" s="42"/>
     </row>
     <row r="50" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B50" s="57" t="s">
-        <v>64</v>
-      </c>
-      <c r="C50" s="58"/>
-      <c r="D50" s="58"/>
-      <c r="E50" s="58"/>
-      <c r="F50" s="58"/>
-      <c r="G50" s="58"/>
-      <c r="H50" s="58"/>
-      <c r="I50" s="58"/>
-      <c r="J50" s="58"/>
-      <c r="K50" s="59"/>
+      <c r="B50" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="C50" s="34"/>
+      <c r="D50" s="34"/>
+      <c r="E50" s="34"/>
+      <c r="F50" s="34"/>
+      <c r="G50" s="34"/>
+      <c r="H50" s="34"/>
+      <c r="I50" s="34"/>
+      <c r="J50" s="34"/>
+      <c r="K50" s="35"/>
     </row>
     <row r="51" spans="2:27" ht="18" customHeight="1">
       <c r="B51" s="15"/>
@@ -2792,10 +2792,10 @@
       <c r="K52" s="20"/>
     </row>
     <row r="53" spans="2:27" ht="42" customHeight="1">
-      <c r="B53" s="52"/>
-      <c r="C53" s="53"/>
-      <c r="D53" s="53"/>
-      <c r="E53" s="53"/>
+      <c r="B53" s="62"/>
+      <c r="C53" s="52"/>
+      <c r="D53" s="52"/>
+      <c r="E53" s="52"/>
       <c r="F53" s="21"/>
       <c r="G53" s="22"/>
       <c r="H53" s="22"/>
@@ -2804,12 +2804,12 @@
       <c r="K53" s="23"/>
     </row>
     <row r="54" spans="2:27" ht="41.45" customHeight="1">
-      <c r="B54" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="C54" s="27"/>
-      <c r="D54" s="27"/>
-      <c r="E54" s="27"/>
+      <c r="B54" s="65" t="s">
+        <v>62</v>
+      </c>
+      <c r="C54" s="50"/>
+      <c r="D54" s="50"/>
+      <c r="E54" s="50"/>
       <c r="F54" s="21"/>
       <c r="G54" s="22"/>
       <c r="H54" s="22"/>
@@ -2846,18 +2846,18 @@
       <c r="AA55" s="10"/>
     </row>
     <row r="56" spans="2:27" ht="22.5" customHeight="1">
-      <c r="B56" s="47" t="s">
-        <v>66</v>
-      </c>
-      <c r="C56" s="48"/>
-      <c r="D56" s="48"/>
-      <c r="E56" s="48"/>
-      <c r="F56" s="48"/>
-      <c r="G56" s="48"/>
-      <c r="H56" s="48"/>
-      <c r="I56" s="48"/>
-      <c r="J56" s="48"/>
-      <c r="K56" s="49"/>
+      <c r="B56" s="59" t="s">
+        <v>63</v>
+      </c>
+      <c r="C56" s="60"/>
+      <c r="D56" s="60"/>
+      <c r="E56" s="60"/>
+      <c r="F56" s="60"/>
+      <c r="G56" s="60"/>
+      <c r="H56" s="60"/>
+      <c r="I56" s="60"/>
+      <c r="J56" s="60"/>
+      <c r="K56" s="61"/>
     </row>
     <row r="57" spans="2:27" ht="6.75" customHeight="1">
       <c r="B57" s="11"/>
@@ -3900,6 +3900,65 @@
     <row r="996" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="75">
+    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="C43:K43"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="H22:H24"/>
+    <mergeCell ref="D16:K16"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="C46:K46"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B20:K20"/>
+    <mergeCell ref="B40:K40"/>
+    <mergeCell ref="B31:K31"/>
+    <mergeCell ref="C42:K42"/>
+    <mergeCell ref="B26:C28"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:K10"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="F35:K35"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B12:C13"/>
+    <mergeCell ref="D15:K15"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="G12:H13"/>
+    <mergeCell ref="D17:K17"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="D28:G28"/>
+    <mergeCell ref="D11:K11"/>
+    <mergeCell ref="B56:K56"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="C44:K44"/>
+    <mergeCell ref="C47:K47"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B33:K33"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="F38:K38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="F36:K36"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="B22:C24"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="K26:K28"/>
+    <mergeCell ref="D14:K14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D12:F13"/>
+    <mergeCell ref="B14:C14"/>
     <mergeCell ref="C48:K48"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="H21:I21"/>
@@ -3916,65 +3975,6 @@
     <mergeCell ref="J21:K21"/>
     <mergeCell ref="K22:K24"/>
     <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D14:K14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D12:F13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="F36:K36"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="B22:C24"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="K26:K28"/>
-    <mergeCell ref="B56:K56"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="C44:K44"/>
-    <mergeCell ref="C47:K47"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="B33:K33"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="F38:K38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B53:E53"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:K10"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="F35:K35"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B12:C13"/>
-    <mergeCell ref="D15:K15"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="G12:H13"/>
-    <mergeCell ref="D17:K17"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="D28:G28"/>
-    <mergeCell ref="D11:K11"/>
-    <mergeCell ref="B54:E54"/>
-    <mergeCell ref="C43:K43"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="H22:H24"/>
-    <mergeCell ref="D16:K16"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="C46:K46"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B20:K20"/>
-    <mergeCell ref="B40:K40"/>
-    <mergeCell ref="B31:K31"/>
-    <mergeCell ref="C42:K42"/>
-    <mergeCell ref="B26:C28"/>
-    <mergeCell ref="D25:G25"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.78740157480314965" bottom="0.78740157480314965" header="0" footer="0"/>
@@ -4034,7 +4034,7 @@
         <v>0</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="14.45" customHeight="1">
@@ -4048,67 +4048,67 @@
         <v>10</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="H3" s="14" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="H4" s="14" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
       <c r="H5" s="14" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
       <c r="H6" s="14" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1">
       <c r="H7" s="14" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1">
       <c r="H8" s="14" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1">
       <c r="H9" s="14" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1">
       <c r="H10" s="14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
       <c r="H11" s="14" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
       <c r="H12" s="14" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15" customHeight="1">
       <c r="H13" s="14" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
       <c r="H14" s="14" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>